<commit_message>
PCB rev.2: 120x61mm, square notch, front-mounted display connector, gold round-button SELECT/START
- board height 85 -> 61 mm; controls re-centered (D-pad left, A/B right,
  SELECT/START below A/B); mounting holes, battery/speaker connectors and
  bottom passives repacked; DRC clean, ~190 stitching vias re-placed
- FPC notch is now square and shallow (26 x 2.5 mm); J3 moved to the FRONT
  (mouth toward the display) so the flat cable inserts straight with no
  fold and no through-board pass -> straight 1:1 pin mapping restored
- SELECT/START switched to XKB TS-1187A-B-A-B (C318884, Basic, gold round
  button) wired diagonally (pairing-safe)
- fab outputs, BOM, pick-and-place and EasyEDA project source regenerated

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/fab/GameFive_BOM.xlsx
+++ b/fab/GameFive_BOM.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="155" uniqueCount="101">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="155" uniqueCount="100">
   <si>
     <t>Supplier</t>
   </si>
@@ -244,16 +244,13 @@
     <t>12</t>
   </si>
   <si>
-    <t>GT-TC155C-H0060-L50.1</t>
-  </si>
-  <si>
-    <t>G-Switch(品赞)</t>
-  </si>
-  <si>
-    <t>GT-TC155C-H0060-L50</t>
-  </si>
-  <si>
-    <t>SW-SMD_4P-G-SWITCH-GT-TC155C-H0060-L50</t>
+    <t>TS-1187A-B-A-B.1</t>
+  </si>
+  <si>
+    <t>TS-1187A-B-A-B</t>
+  </si>
+  <si>
+    <t>SW-SMD_4P-L5.1-W5.1-P3.70-LS6.5-TL_H1.5</t>
   </si>
   <si>
     <t>SW7,SW8</t>
@@ -1120,28 +1117,28 @@
         <v>77</v>
       </c>
       <c r="C14" t="s">
+        <v>40</v>
+      </c>
+      <c r="D14" t="s">
         <v>78</v>
       </c>
-      <c r="D14" t="s">
+      <c r="E14" t="s">
+        <v>14</v>
+      </c>
+      <c r="F14" t="s">
         <v>79</v>
       </c>
-      <c r="E14" t="s">
-        <v>14</v>
-      </c>
-      <c r="F14" t="s">
+      <c r="G14" t="s">
         <v>80</v>
       </c>
-      <c r="G14" t="s">
-        <v>81</v>
-      </c>
       <c r="H14" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="I14">
         <v>2</v>
       </c>
       <c r="J14" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
     </row>
     <row r="15" spans="1:10" x14ac:dyDescent="0.25">
@@ -1149,31 +1146,31 @@
         <v>10</v>
       </c>
       <c r="B15" t="s">
+        <v>82</v>
+      </c>
+      <c r="C15" t="s">
         <v>83</v>
       </c>
-      <c r="C15" t="s">
+      <c r="D15" t="s">
         <v>84</v>
       </c>
-      <c r="D15" t="s">
+      <c r="E15" t="s">
+        <v>14</v>
+      </c>
+      <c r="F15" t="s">
         <v>85</v>
       </c>
-      <c r="E15" t="s">
-        <v>14</v>
-      </c>
-      <c r="F15" t="s">
+      <c r="G15" t="s">
         <v>86</v>
       </c>
-      <c r="G15" t="s">
-        <v>87</v>
-      </c>
       <c r="H15" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="I15">
         <v>1</v>
       </c>
       <c r="J15" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.25">
@@ -1181,31 +1178,31 @@
         <v>10</v>
       </c>
       <c r="B16" t="s">
+        <v>88</v>
+      </c>
+      <c r="C16" t="s">
         <v>89</v>
       </c>
-      <c r="C16" t="s">
+      <c r="D16" t="s">
         <v>90</v>
       </c>
-      <c r="D16" t="s">
+      <c r="E16" t="s">
+        <v>14</v>
+      </c>
+      <c r="F16" t="s">
         <v>91</v>
       </c>
-      <c r="E16" t="s">
-        <v>14</v>
-      </c>
-      <c r="F16" t="s">
+      <c r="G16" t="s">
         <v>92</v>
       </c>
-      <c r="G16" t="s">
-        <v>93</v>
-      </c>
       <c r="H16" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="I16">
         <v>1</v>
       </c>
       <c r="J16" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
     </row>
     <row r="17" spans="1:10" x14ac:dyDescent="0.25">
@@ -1213,31 +1210,31 @@
         <v>10</v>
       </c>
       <c r="B17" t="s">
+        <v>94</v>
+      </c>
+      <c r="C17" t="s">
         <v>95</v>
       </c>
-      <c r="C17" t="s">
+      <c r="D17" t="s">
         <v>96</v>
       </c>
-      <c r="D17" t="s">
+      <c r="E17" t="s">
+        <v>14</v>
+      </c>
+      <c r="F17" t="s">
         <v>97</v>
       </c>
-      <c r="E17" t="s">
-        <v>14</v>
-      </c>
-      <c r="F17" t="s">
+      <c r="G17" t="s">
         <v>98</v>
       </c>
-      <c r="G17" t="s">
-        <v>99</v>
-      </c>
       <c r="H17" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="I17">
         <v>1</v>
       </c>
       <c r="J17" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
     </row>
     <row r="18" spans="1:1" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
PCB rev.2c: drop the speaker circuit for now; display connector lower
- removed U3 (MAX98357A), J2 (speaker JST) and R12 (SD_MODE pull-up);
  XIAO I2S pins stay reserved for a future audio add-on
- J3 moved further down under the panel (contact row ~15 mm below the
  module top edge, within the folded tail's reach)
- rerouted, 194 stitching vias, DRC clean; fab/BOM/PnP/EasyEDA source updated

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/fab/GameFive_BOM.xlsx
+++ b/fab/GameFive_BOM.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="155" uniqueCount="100">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="137" uniqueCount="88">
   <si>
     <t>Supplier</t>
   </si>
@@ -112,205 +112,169 @@
     <t>4</t>
   </si>
   <si>
-    <t>PH-2PS.1</t>
-  </si>
-  <si>
-    <t>DEALON(德艺隆)</t>
-  </si>
-  <si>
-    <t>PH-2PS</t>
-  </si>
-  <si>
-    <t>CONN-SMD_2P-P2.00_DEALON_PH-2PS</t>
-  </si>
-  <si>
-    <t>J2</t>
+    <t>X05A20L12T.1</t>
+  </si>
+  <si>
+    <t>XKB Connection(中国星坤)</t>
+  </si>
+  <si>
+    <t>X05A20L12T</t>
+  </si>
+  <si>
+    <t>FFC-SMD_12P-P0.50_X05A20L12T</t>
+  </si>
+  <si>
+    <t>J3</t>
   </si>
   <si>
     <t>5</t>
   </si>
   <si>
-    <t>X05A20L12T.1</t>
-  </si>
-  <si>
-    <t>XKB Connection(中国星坤)</t>
-  </si>
-  <si>
-    <t>X05A20L12T</t>
-  </si>
-  <si>
-    <t>FFC-SMD_12P-P0.50_X05A20L12T</t>
-  </si>
-  <si>
-    <t>J3</t>
+    <t>SI2302_C2938373.1</t>
+  </si>
+  <si>
+    <t>GOODWORK(固得沃克)</t>
+  </si>
+  <si>
+    <t>SI2302</t>
+  </si>
+  <si>
+    <t>SOT-23_L2.9-W1.3-P1.90-LS2.4-BR</t>
+  </si>
+  <si>
+    <t>Q1</t>
   </si>
   <si>
     <t>6</t>
   </si>
   <si>
-    <t>SI2302_C2938373.1</t>
-  </si>
-  <si>
-    <t>GOODWORK(固得沃克)</t>
-  </si>
-  <si>
-    <t>SI2302</t>
-  </si>
-  <si>
-    <t>SOT-23_L2.9-W1.3-P1.90-LS2.4-BR</t>
-  </si>
-  <si>
-    <t>Q1</t>
+    <t>C191123</t>
+  </si>
+  <si>
+    <t>PANASONIC</t>
+  </si>
+  <si>
+    <t>ERJ2RKF1002X</t>
+  </si>
+  <si>
+    <t>R0402</t>
+  </si>
+  <si>
+    <t>R1,R2,R3,R4,R5,R6,R7,R8</t>
   </si>
   <si>
     <t>7</t>
   </si>
   <si>
-    <t>C191123</t>
-  </si>
-  <si>
-    <t>PANASONIC</t>
-  </si>
-  <si>
-    <t>ERJ2RKF1002X</t>
-  </si>
-  <si>
-    <t>R0402</t>
-  </si>
-  <si>
-    <t>R1,R2,R3,R4,R5,R6,R7,R8</t>
+    <t>0805W8F220JT5E.1</t>
+  </si>
+  <si>
+    <t>UNI-ROYAL(厚声)</t>
+  </si>
+  <si>
+    <t>0805W8F220JT5E</t>
+  </si>
+  <si>
+    <t>R0805</t>
+  </si>
+  <si>
+    <t>R9</t>
   </si>
   <si>
     <t>8</t>
   </si>
   <si>
-    <t>0805W8F220JT5E.1</t>
-  </si>
-  <si>
-    <t>UNI-ROYAL(厚声)</t>
-  </si>
-  <si>
-    <t>0805W8F220JT5E</t>
-  </si>
-  <si>
-    <t>R0805</t>
-  </si>
-  <si>
-    <t>R9</t>
+    <t>0402WGF1000TCE.1</t>
+  </si>
+  <si>
+    <t>0402WGF1000TCE</t>
+  </si>
+  <si>
+    <t>R10</t>
   </si>
   <si>
     <t>9</t>
   </si>
   <si>
-    <t>0402WGF1000TCE.1</t>
-  </si>
-  <si>
-    <t>0402WGF1000TCE</t>
-  </si>
-  <si>
-    <t>R10</t>
+    <t>0402WGF1003TCE.1</t>
+  </si>
+  <si>
+    <t>0402WGF1003TCE</t>
+  </si>
+  <si>
+    <t>R11</t>
   </si>
   <si>
     <t>10</t>
   </si>
   <si>
-    <t>0402WGF1003TCE.1</t>
-  </si>
-  <si>
-    <t>0402WGF1003TCE</t>
-  </si>
-  <si>
-    <t>R11,R12</t>
+    <t>EVQQ1D06M.1</t>
+  </si>
+  <si>
+    <t>PANASONIC(松下)</t>
+  </si>
+  <si>
+    <t>EVQQ1D06M</t>
+  </si>
+  <si>
+    <t>SW-SMD_4P-L10.0-W8.6-P4.50-LS10.0</t>
+  </si>
+  <si>
+    <t>SW1,SW2,SW3,SW4,SW5,SW6</t>
   </si>
   <si>
     <t>11</t>
   </si>
   <si>
-    <t>EVQQ1D06M.1</t>
-  </si>
-  <si>
-    <t>PANASONIC(松下)</t>
-  </si>
-  <si>
-    <t>EVQQ1D06M</t>
-  </si>
-  <si>
-    <t>SW-SMD_4P-L10.0-W8.6-P4.50-LS10.0</t>
-  </si>
-  <si>
-    <t>SW1,SW2,SW3,SW4,SW5,SW6</t>
+    <t>TS-1187A-B-A-B.1</t>
+  </si>
+  <si>
+    <t>TS-1187A-B-A-B</t>
+  </si>
+  <si>
+    <t>SW-SMD_4P-L5.1-W5.1-P3.70-LS6.5-TL_H1.5</t>
+  </si>
+  <si>
+    <t>SW7,SW8</t>
   </si>
   <si>
     <t>12</t>
   </si>
   <si>
-    <t>TS-1187A-B-A-B.1</t>
-  </si>
-  <si>
-    <t>TS-1187A-B-A-B</t>
-  </si>
-  <si>
-    <t>SW-SMD_4P-L5.1-W5.1-P3.70-LS6.5-TL_H1.5</t>
-  </si>
-  <si>
-    <t>SW7,SW8</t>
+    <t>C9900154951</t>
+  </si>
+  <si>
+    <t>JLCPCB</t>
+  </si>
+  <si>
+    <t>XIAO ESP32S3</t>
+  </si>
+  <si>
+    <t>COMM-SMD_L21.1-W17.8-P2.54_113991114_XIAO-ESP32-S3</t>
+  </si>
+  <si>
+    <t>U1</t>
   </si>
   <si>
     <t>13</t>
   </si>
   <si>
-    <t>C9900154951</t>
-  </si>
-  <si>
-    <t>JLCPCB</t>
-  </si>
-  <si>
-    <t>XIAO ESP32S3</t>
-  </si>
-  <si>
-    <t>COMM-SMD_L21.1-W17.8-P2.54_113991114_XIAO-ESP32-S3</t>
-  </si>
-  <si>
-    <t>U1</t>
+    <t>SN74HC165DR.1</t>
+  </si>
+  <si>
+    <t>TI(德州仪器)</t>
+  </si>
+  <si>
+    <t>SN74HC165DR</t>
+  </si>
+  <si>
+    <t>SOP-16_L10.0-W3.9-P1.27-LS6.0-BL</t>
+  </si>
+  <si>
+    <t>U2</t>
   </si>
   <si>
     <t>14</t>
-  </si>
-  <si>
-    <t>SN74HC165DR.1</t>
-  </si>
-  <si>
-    <t>TI(德州仪器)</t>
-  </si>
-  <si>
-    <t>SN74HC165DR</t>
-  </si>
-  <si>
-    <t>SOP-16_L10.0-W3.9-P1.27-LS6.0-BL</t>
-  </si>
-  <si>
-    <t>U2</t>
-  </si>
-  <si>
-    <t>15</t>
-  </si>
-  <si>
-    <t>MAX98357AETE+T.1</t>
-  </si>
-  <si>
-    <t>ADI(亚德诺)/MAXIM(美信)</t>
-  </si>
-  <si>
-    <t>MAX98357AETE+T</t>
-  </si>
-  <si>
-    <t>TQFN-16_L3.0-W3.0-P0.50-BL-EP1.5</t>
-  </si>
-  <si>
-    <t>U3</t>
-  </si>
-  <si>
-    <t>16</t>
   </si>
 </sst>
 </file>
@@ -687,7 +651,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:J18"/>
+  <dimension ref="A1:J16"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="10" width="20" customWidth="1"/>
@@ -943,7 +907,7 @@
         <v>47</v>
       </c>
       <c r="I8">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="J8" t="s">
         <v>50</v>
@@ -975,7 +939,7 @@
         <v>53</v>
       </c>
       <c r="I9">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="J9" t="s">
         <v>56</v>
@@ -989,28 +953,28 @@
         <v>57</v>
       </c>
       <c r="C10" t="s">
+        <v>52</v>
+      </c>
+      <c r="D10" t="s">
         <v>58</v>
       </c>
-      <c r="D10" t="s">
+      <c r="E10" t="s">
+        <v>14</v>
+      </c>
+      <c r="F10" t="s">
+        <v>48</v>
+      </c>
+      <c r="G10" t="s">
         <v>59</v>
       </c>
-      <c r="E10" t="s">
-        <v>14</v>
-      </c>
-      <c r="F10" t="s">
-        <v>60</v>
-      </c>
-      <c r="G10" t="s">
-        <v>61</v>
-      </c>
       <c r="H10" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="I10">
         <v>1</v>
       </c>
       <c r="J10" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.25">
@@ -1018,31 +982,31 @@
         <v>10</v>
       </c>
       <c r="B11" t="s">
+        <v>61</v>
+      </c>
+      <c r="C11" t="s">
+        <v>52</v>
+      </c>
+      <c r="D11" t="s">
+        <v>62</v>
+      </c>
+      <c r="E11" t="s">
+        <v>14</v>
+      </c>
+      <c r="F11" t="s">
+        <v>48</v>
+      </c>
+      <c r="G11" t="s">
         <v>63</v>
       </c>
-      <c r="C11" t="s">
-        <v>58</v>
-      </c>
-      <c r="D11" t="s">
-        <v>64</v>
-      </c>
-      <c r="E11" t="s">
-        <v>14</v>
-      </c>
-      <c r="F11" t="s">
-        <v>54</v>
-      </c>
-      <c r="G11" t="s">
-        <v>65</v>
-      </c>
       <c r="H11" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="I11">
         <v>1</v>
       </c>
       <c r="J11" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.25">
@@ -1050,28 +1014,28 @@
         <v>10</v>
       </c>
       <c r="B12" t="s">
+        <v>65</v>
+      </c>
+      <c r="C12" t="s">
+        <v>66</v>
+      </c>
+      <c r="D12" t="s">
         <v>67</v>
       </c>
-      <c r="C12" t="s">
-        <v>58</v>
-      </c>
-      <c r="D12" t="s">
+      <c r="E12" t="s">
+        <v>14</v>
+      </c>
+      <c r="F12" t="s">
         <v>68</v>
-      </c>
-      <c r="E12" t="s">
-        <v>14</v>
-      </c>
-      <c r="F12" t="s">
-        <v>54</v>
       </c>
       <c r="G12" t="s">
         <v>69</v>
       </c>
       <c r="H12" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="I12">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="J12" t="s">
         <v>70</v>
@@ -1085,28 +1049,28 @@
         <v>71</v>
       </c>
       <c r="C13" t="s">
+        <v>34</v>
+      </c>
+      <c r="D13" t="s">
         <v>72</v>
       </c>
-      <c r="D13" t="s">
+      <c r="E13" t="s">
+        <v>14</v>
+      </c>
+      <c r="F13" t="s">
         <v>73</v>
       </c>
-      <c r="E13" t="s">
-        <v>14</v>
-      </c>
-      <c r="F13" t="s">
+      <c r="G13" t="s">
         <v>74</v>
       </c>
-      <c r="G13" t="s">
+      <c r="H13" t="s">
+        <v>72</v>
+      </c>
+      <c r="I13">
+        <v>2</v>
+      </c>
+      <c r="J13" t="s">
         <v>75</v>
-      </c>
-      <c r="H13" t="s">
-        <v>73</v>
-      </c>
-      <c r="I13">
-        <v>6</v>
-      </c>
-      <c r="J13" t="s">
-        <v>76</v>
       </c>
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.25">
@@ -1114,10 +1078,10 @@
         <v>10</v>
       </c>
       <c r="B14" t="s">
+        <v>76</v>
+      </c>
+      <c r="C14" t="s">
         <v>77</v>
-      </c>
-      <c r="C14" t="s">
-        <v>40</v>
       </c>
       <c r="D14" t="s">
         <v>78</v>
@@ -1135,7 +1099,7 @@
         <v>78</v>
       </c>
       <c r="I14">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J14" t="s">
         <v>81</v>
@@ -1173,72 +1137,8 @@
         <v>87</v>
       </c>
     </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>10</v>
-      </c>
-      <c r="B16" t="s">
-        <v>88</v>
-      </c>
-      <c r="C16" t="s">
-        <v>89</v>
-      </c>
-      <c r="D16" t="s">
-        <v>90</v>
-      </c>
-      <c r="E16" t="s">
-        <v>14</v>
-      </c>
-      <c r="F16" t="s">
-        <v>91</v>
-      </c>
-      <c r="G16" t="s">
-        <v>92</v>
-      </c>
-      <c r="H16" t="s">
-        <v>90</v>
-      </c>
-      <c r="I16">
-        <v>1</v>
-      </c>
-      <c r="J16" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="17" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A17" t="s">
-        <v>10</v>
-      </c>
-      <c r="B17" t="s">
-        <v>94</v>
-      </c>
-      <c r="C17" t="s">
-        <v>95</v>
-      </c>
-      <c r="D17" t="s">
-        <v>96</v>
-      </c>
-      <c r="E17" t="s">
-        <v>14</v>
-      </c>
-      <c r="F17" t="s">
-        <v>97</v>
-      </c>
-      <c r="G17" t="s">
-        <v>98</v>
-      </c>
-      <c r="H17" t="s">
-        <v>96</v>
-      </c>
-      <c r="I17">
-        <v>1</v>
-      </c>
-      <c r="J17" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="18" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A18" t="s">
         <v>14</v>
       </c>
     </row>

</xml_diff>

<commit_message>
PCB rev.2e: SELECT/START to bottom-center with taller switches; A/B lowered
- SELECT/START moved below the display (GameBoy-style pair) and switched
  to XKB TS-1187A-C-H-B (C528025) with a 4 mm gold round button
- display frame raised (top edge 3 mm from board top) to make room;
  J3 stays at the user-specified absolute 18.5 mm from the board top
- A/B lowered to y=-1450; labels repositioned
- rerouted, 208 stitching vias, DRC clean; fab/BOM/PnP/EasyEDA source updated

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/fab/GameFive_BOM.xlsx
+++ b/fab/GameFive_BOM.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="137" uniqueCount="88">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="137" uniqueCount="89">
   <si>
     <t>Supplier</t>
   </si>
@@ -226,13 +226,16 @@
     <t>11</t>
   </si>
   <si>
-    <t>TS-1187A-B-A-B.1</t>
-  </si>
-  <si>
-    <t>TS-1187A-B-A-B</t>
-  </si>
-  <si>
-    <t>SW-SMD_4P-L5.1-W5.1-P3.70-LS6.5-TL_H1.5</t>
+    <t>TS-1187A-C-H-B.1</t>
+  </si>
+  <si>
+    <t>XKB Connectivity(中国星坤)</t>
+  </si>
+  <si>
+    <t>TS-1187A-C-H-B</t>
+  </si>
+  <si>
+    <t>SW-SMD_4P-L5.1-W5.1-P3.70-LS6.5-TL_H4.0</t>
   </si>
   <si>
     <t>SW7,SW8</t>
@@ -1049,28 +1052,28 @@
         <v>71</v>
       </c>
       <c r="C13" t="s">
-        <v>34</v>
+        <v>72</v>
       </c>
       <c r="D13" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="E13" t="s">
         <v>14</v>
       </c>
       <c r="F13" t="s">
+        <v>74</v>
+      </c>
+      <c r="G13" t="s">
+        <v>75</v>
+      </c>
+      <c r="H13" t="s">
         <v>73</v>
-      </c>
-      <c r="G13" t="s">
-        <v>74</v>
-      </c>
-      <c r="H13" t="s">
-        <v>72</v>
       </c>
       <c r="I13">
         <v>2</v>
       </c>
       <c r="J13" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.25">
@@ -1078,31 +1081,31 @@
         <v>10</v>
       </c>
       <c r="B14" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="C14" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="D14" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="E14" t="s">
         <v>14</v>
       </c>
       <c r="F14" t="s">
+        <v>80</v>
+      </c>
+      <c r="G14" t="s">
+        <v>81</v>
+      </c>
+      <c r="H14" t="s">
         <v>79</v>
-      </c>
-      <c r="G14" t="s">
-        <v>80</v>
-      </c>
-      <c r="H14" t="s">
-        <v>78</v>
       </c>
       <c r="I14">
         <v>1</v>
       </c>
       <c r="J14" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
     </row>
     <row r="15" spans="1:10" x14ac:dyDescent="0.25">
@@ -1110,31 +1113,31 @@
         <v>10</v>
       </c>
       <c r="B15" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="C15" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="D15" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="E15" t="s">
         <v>14</v>
       </c>
       <c r="F15" t="s">
+        <v>86</v>
+      </c>
+      <c r="G15" t="s">
+        <v>87</v>
+      </c>
+      <c r="H15" t="s">
         <v>85</v>
-      </c>
-      <c r="G15" t="s">
-        <v>86</v>
-      </c>
-      <c r="H15" t="s">
-        <v>84</v>
       </c>
       <c r="I15">
         <v>1</v>
       </c>
       <c r="J15" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
     </row>
     <row r="16" spans="1:1" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
PCB rev.2f: Omron B3F-1025 SELECT/START (crisp THT click), XIAO raised
- SELECT/START switched to Omron B3F-1025 (C726009): 6x6 through-hole,
  orange round button, 2.55 N crisp tactile click, wired diagonally
- display frame raised to 1.5 mm from the top edge and J3 moved with it,
  preserving the user-measured connector-to-module relation (housing top
  edge 10.4 mm below the module top edge); bottom strip now fits the 6 mm
  switch bodies with clean outline clearances
- XIAO moved up ~5 mm (USB-C stays on the right edge); battery connector
  relocated to clear the new through-hole pins
- rerouted, 221 stitching vias, DRC clean; fab/BOM/PnP/EasyEDA source updated

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/fab/GameFive_BOM.xlsx
+++ b/fab/GameFive_BOM.xlsx
@@ -226,16 +226,16 @@
     <t>11</t>
   </si>
   <si>
-    <t>TS-1187A-C-H-B.1</t>
-  </si>
-  <si>
-    <t>XKB Connectivity(中国星坤)</t>
-  </si>
-  <si>
-    <t>TS-1187A-C-H-B</t>
-  </si>
-  <si>
-    <t>SW-SMD_4P-L5.1-W5.1-P3.70-LS6.5-TL_H4.0</t>
+    <t>B3F-1025.1</t>
+  </si>
+  <si>
+    <t>OMRON(欧姆龙)</t>
+  </si>
+  <si>
+    <t>B3F-1025</t>
+  </si>
+  <si>
+    <t>SW-TH_4P-L6.2-W6.2-P4.50-LS6.5</t>
   </si>
   <si>
     <t>SW7,SW8</t>

</xml_diff>